<commit_message>
violin html output added
</commit_message>
<xml_diff>
--- a/plotting_and_statistics_script_with_demo_data/output_files_of_py_script/2025-12-03 08_15_00_TEMP_LOG_demo_data.xlsx
+++ b/plotting_and_statistics_script_with_demo_data/output_files_of_py_script/2025-12-03 08_15_00_TEMP_LOG_demo_data.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,27 +421,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Logger-id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Vbatt</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Date_time</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>TMP1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>TMP2</t>
         </is>
@@ -468,7 +456,7 @@
       <c r="B2" t="n">
         <v>3944</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="1" t="n">
         <v>45993.64236111111</v>
       </c>
       <c r="D2" t="n">
@@ -487,7 +475,7 @@
       <c r="B3" t="n">
         <v>3944</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="1" t="n">
         <v>45993.64583333334</v>
       </c>
       <c r="D3" t="n">
@@ -506,7 +494,7 @@
       <c r="B4" t="n">
         <v>3944</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="1" t="n">
         <v>45993.64930555555</v>
       </c>
       <c r="D4" t="n">
@@ -525,7 +513,7 @@
       <c r="B5" t="n">
         <v>3944</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="1" t="n">
         <v>45993.65277777778</v>
       </c>
       <c r="D5" t="n">
@@ -544,7 +532,7 @@
       <c r="B6" t="n">
         <v>3944</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="1" t="n">
         <v>45993.65972222222</v>
       </c>
       <c r="D6" t="n">
@@ -563,7 +551,7 @@
       <c r="B7" t="n">
         <v>3944</v>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="1" t="n">
         <v>45993.66319444445</v>
       </c>
       <c r="D7" t="n">
@@ -582,7 +570,7 @@
       <c r="B8" t="n">
         <v>3944</v>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="1" t="n">
         <v>45993.66666666666</v>
       </c>
       <c r="D8" t="n">
@@ -601,7 +589,7 @@
       <c r="B9" t="n">
         <v>3944</v>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="1" t="n">
         <v>45993.67013888889</v>
       </c>
       <c r="D9" t="n">
@@ -620,7 +608,7 @@
       <c r="B10" t="n">
         <v>3944</v>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="1" t="n">
         <v>45993.67361111111</v>
       </c>
       <c r="D10" t="n">
@@ -639,7 +627,7 @@
       <c r="B11" t="n">
         <v>3944</v>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" s="1" t="n">
         <v>45993.67708333334</v>
       </c>
       <c r="D11" t="n">
@@ -658,7 +646,7 @@
       <c r="B12" t="n">
         <v>3944</v>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C12" s="1" t="n">
         <v>45993.68055555555</v>
       </c>
       <c r="D12" t="n">
@@ -677,7 +665,7 @@
       <c r="B13" t="n">
         <v>3944</v>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="C13" s="1" t="n">
         <v>45993.68402777778</v>
       </c>
       <c r="D13" t="n">
@@ -696,7 +684,7 @@
       <c r="B14" t="n">
         <v>3944</v>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C14" s="1" t="n">
         <v>45993.6875</v>
       </c>
       <c r="D14" t="n">
@@ -715,7 +703,7 @@
       <c r="B15" t="n">
         <v>3944</v>
       </c>
-      <c r="C15" s="2" t="n">
+      <c r="C15" s="1" t="n">
         <v>45993.69097222222</v>
       </c>
       <c r="D15" t="n">
@@ -734,7 +722,7 @@
       <c r="B16" t="n">
         <v>3944</v>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="C16" s="1" t="n">
         <v>45993.69444444445</v>
       </c>
       <c r="D16" t="n">
@@ -753,7 +741,7 @@
       <c r="B17" t="n">
         <v>3944</v>
       </c>
-      <c r="C17" s="2" t="n">
+      <c r="C17" s="1" t="n">
         <v>45993.69791666666</v>
       </c>
       <c r="D17" t="n">
@@ -772,7 +760,7 @@
       <c r="B18" t="n">
         <v>3944</v>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="C18" s="1" t="n">
         <v>45993.70138888889</v>
       </c>
       <c r="D18" t="n">
@@ -791,7 +779,7 @@
       <c r="B19" t="n">
         <v>3944</v>
       </c>
-      <c r="C19" s="2" t="n">
+      <c r="C19" s="1" t="n">
         <v>45993.70486111111</v>
       </c>
       <c r="D19" t="n">
@@ -810,7 +798,7 @@
       <c r="B20" t="n">
         <v>3944</v>
       </c>
-      <c r="C20" s="2" t="n">
+      <c r="C20" s="1" t="n">
         <v>45993.70833333334</v>
       </c>
       <c r="D20" t="n">
@@ -829,7 +817,7 @@
       <c r="B21" t="n">
         <v>3944</v>
       </c>
-      <c r="C21" s="2" t="n">
+      <c r="C21" s="1" t="n">
         <v>45993.71180555555</v>
       </c>
       <c r="D21" t="n">
@@ -848,7 +836,7 @@
       <c r="B22" t="n">
         <v>3944</v>
       </c>
-      <c r="C22" s="2" t="n">
+      <c r="C22" s="1" t="n">
         <v>45993.71527777778</v>
       </c>
       <c r="D22" t="n">
@@ -867,7 +855,7 @@
       <c r="B23" t="n">
         <v>3944</v>
       </c>
-      <c r="C23" s="2" t="n">
+      <c r="C23" s="1" t="n">
         <v>45993.71875</v>
       </c>
       <c r="D23" t="n">
@@ -886,7 +874,7 @@
       <c r="B24" t="n">
         <v>3944</v>
       </c>
-      <c r="C24" s="2" t="n">
+      <c r="C24" s="1" t="n">
         <v>45993.72222222222</v>
       </c>
       <c r="D24" t="n">
@@ -905,7 +893,7 @@
       <c r="B25" t="n">
         <v>3944</v>
       </c>
-      <c r="C25" s="2" t="n">
+      <c r="C25" s="1" t="n">
         <v>45993.72569444445</v>
       </c>
       <c r="D25" t="n">
@@ -924,7 +912,7 @@
       <c r="B26" t="n">
         <v>3944</v>
       </c>
-      <c r="C26" s="2" t="n">
+      <c r="C26" s="1" t="n">
         <v>45993.72916666666</v>
       </c>
       <c r="D26" t="n">
@@ -943,7 +931,7 @@
       <c r="B27" t="n">
         <v>3944</v>
       </c>
-      <c r="C27" s="2" t="n">
+      <c r="C27" s="1" t="n">
         <v>45993.73263888889</v>
       </c>
       <c r="D27" t="n">
@@ -962,7 +950,7 @@
       <c r="B28" t="n">
         <v>3944</v>
       </c>
-      <c r="C28" s="2" t="n">
+      <c r="C28" s="1" t="n">
         <v>45993.73611111111</v>
       </c>
       <c r="D28" t="n">
@@ -981,7 +969,7 @@
       <c r="B29" t="n">
         <v>3944</v>
       </c>
-      <c r="C29" s="2" t="n">
+      <c r="C29" s="1" t="n">
         <v>45993.73958333334</v>
       </c>
       <c r="D29" t="n">
@@ -1000,7 +988,7 @@
       <c r="B30" t="n">
         <v>3944</v>
       </c>
-      <c r="C30" s="2" t="n">
+      <c r="C30" s="1" t="n">
         <v>45993.74305555555</v>
       </c>
       <c r="D30" t="n">
@@ -1019,7 +1007,7 @@
       <c r="B31" t="n">
         <v>3944</v>
       </c>
-      <c r="C31" s="2" t="n">
+      <c r="C31" s="1" t="n">
         <v>45993.74652777778</v>
       </c>
       <c r="D31" t="n">
@@ -1038,7 +1026,7 @@
       <c r="B32" t="n">
         <v>3944</v>
       </c>
-      <c r="C32" s="2" t="n">
+      <c r="C32" s="1" t="n">
         <v>45993.75</v>
       </c>
       <c r="D32" t="n">
@@ -1057,7 +1045,7 @@
       <c r="B33" t="n">
         <v>3944</v>
       </c>
-      <c r="C33" s="2" t="n">
+      <c r="C33" s="1" t="n">
         <v>45993.75347222222</v>
       </c>
       <c r="D33" t="n">
@@ -1076,7 +1064,7 @@
       <c r="B34" t="n">
         <v>3944</v>
       </c>
-      <c r="C34" s="2" t="n">
+      <c r="C34" s="1" t="n">
         <v>45993.75694444445</v>
       </c>
       <c r="D34" t="n">
@@ -1095,7 +1083,7 @@
       <c r="B35" t="n">
         <v>3944</v>
       </c>
-      <c r="C35" s="2" t="n">
+      <c r="C35" s="1" t="n">
         <v>45993.76041666666</v>
       </c>
       <c r="D35" t="n">
@@ -1114,7 +1102,7 @@
       <c r="B36" t="n">
         <v>3944</v>
       </c>
-      <c r="C36" s="2" t="n">
+      <c r="C36" s="1" t="n">
         <v>45993.76388888889</v>
       </c>
       <c r="D36" t="n">
@@ -1133,7 +1121,7 @@
       <c r="B37" t="n">
         <v>3944</v>
       </c>
-      <c r="C37" s="2" t="n">
+      <c r="C37" s="1" t="n">
         <v>45993.76736111111</v>
       </c>
       <c r="D37" t="n">
@@ -1152,7 +1140,7 @@
       <c r="B38" t="n">
         <v>3944</v>
       </c>
-      <c r="C38" s="2" t="n">
+      <c r="C38" s="1" t="n">
         <v>45993.77083333334</v>
       </c>
       <c r="D38" t="n">
@@ -1171,7 +1159,7 @@
       <c r="B39" t="n">
         <v>3944</v>
       </c>
-      <c r="C39" s="2" t="n">
+      <c r="C39" s="1" t="n">
         <v>45993.77430555555</v>
       </c>
       <c r="D39" t="n">
@@ -1190,7 +1178,7 @@
       <c r="B40" t="n">
         <v>3944</v>
       </c>
-      <c r="C40" s="2" t="n">
+      <c r="C40" s="1" t="n">
         <v>45993.77777777778</v>
       </c>
       <c r="D40" t="n">
@@ -1209,7 +1197,7 @@
       <c r="B41" t="n">
         <v>3944</v>
       </c>
-      <c r="C41" s="2" t="n">
+      <c r="C41" s="1" t="n">
         <v>45993.78125</v>
       </c>
       <c r="D41" t="n">
@@ -1228,7 +1216,7 @@
       <c r="B42" t="n">
         <v>3944</v>
       </c>
-      <c r="C42" s="2" t="n">
+      <c r="C42" s="1" t="n">
         <v>45993.78472222222</v>
       </c>
       <c r="D42" t="n">
@@ -1247,7 +1235,7 @@
       <c r="B43" t="n">
         <v>3944</v>
       </c>
-      <c r="C43" s="2" t="n">
+      <c r="C43" s="1" t="n">
         <v>45993.78819444445</v>
       </c>
       <c r="D43" t="n">
@@ -1266,7 +1254,7 @@
       <c r="B44" t="n">
         <v>3944</v>
       </c>
-      <c r="C44" s="2" t="n">
+      <c r="C44" s="1" t="n">
         <v>45993.79166666666</v>
       </c>
       <c r="D44" t="n">
@@ -1285,7 +1273,7 @@
       <c r="B45" t="n">
         <v>3944</v>
       </c>
-      <c r="C45" s="2" t="n">
+      <c r="C45" s="1" t="n">
         <v>45993.79513888889</v>
       </c>
       <c r="D45" t="n">
@@ -1304,7 +1292,7 @@
       <c r="B46" t="n">
         <v>3944</v>
       </c>
-      <c r="C46" s="2" t="n">
+      <c r="C46" s="1" t="n">
         <v>45993.79861111111</v>
       </c>
       <c r="D46" t="n">
@@ -1323,7 +1311,7 @@
       <c r="B47" t="n">
         <v>3944</v>
       </c>
-      <c r="C47" s="2" t="n">
+      <c r="C47" s="1" t="n">
         <v>45993.80208333334</v>
       </c>
       <c r="D47" t="n">
@@ -1342,7 +1330,7 @@
       <c r="B48" t="n">
         <v>3944</v>
       </c>
-      <c r="C48" s="2" t="n">
+      <c r="C48" s="1" t="n">
         <v>45993.80555555555</v>
       </c>
       <c r="D48" t="n">
@@ -1361,7 +1349,7 @@
       <c r="B49" t="n">
         <v>3944</v>
       </c>
-      <c r="C49" s="2" t="n">
+      <c r="C49" s="1" t="n">
         <v>45993.80902777778</v>
       </c>
       <c r="D49" t="n">
@@ -1380,7 +1368,7 @@
       <c r="B50" t="n">
         <v>3944</v>
       </c>
-      <c r="C50" s="2" t="n">
+      <c r="C50" s="1" t="n">
         <v>45993.8125</v>
       </c>
       <c r="D50" t="n">
@@ -1399,7 +1387,7 @@
       <c r="B51" t="n">
         <v>3944</v>
       </c>
-      <c r="C51" s="2" t="n">
+      <c r="C51" s="1" t="n">
         <v>45993.81597222222</v>
       </c>
       <c r="D51" t="n">
@@ -1418,7 +1406,7 @@
       <c r="B52" t="n">
         <v>3944</v>
       </c>
-      <c r="C52" s="2" t="n">
+      <c r="C52" s="1" t="n">
         <v>45993.81944444445</v>
       </c>
       <c r="D52" t="n">
@@ -1437,7 +1425,7 @@
       <c r="B53" t="n">
         <v>3944</v>
       </c>
-      <c r="C53" s="2" t="n">
+      <c r="C53" s="1" t="n">
         <v>45993.82291666666</v>
       </c>
       <c r="D53" t="n">
@@ -1456,7 +1444,7 @@
       <c r="B54" t="n">
         <v>3944</v>
       </c>
-      <c r="C54" s="2" t="n">
+      <c r="C54" s="1" t="n">
         <v>45993.82638888889</v>
       </c>
       <c r="D54" t="n">
@@ -1475,7 +1463,7 @@
       <c r="B55" t="n">
         <v>3944</v>
       </c>
-      <c r="C55" s="2" t="n">
+      <c r="C55" s="1" t="n">
         <v>45993.82986111111</v>
       </c>
       <c r="D55" t="n">
@@ -1494,7 +1482,7 @@
       <c r="B56" t="n">
         <v>3944</v>
       </c>
-      <c r="C56" s="2" t="n">
+      <c r="C56" s="1" t="n">
         <v>45993.83333333334</v>
       </c>
       <c r="D56" t="n">
@@ -1513,7 +1501,7 @@
       <c r="B57" t="n">
         <v>3944</v>
       </c>
-      <c r="C57" s="2" t="n">
+      <c r="C57" s="1" t="n">
         <v>45993.83680555555</v>
       </c>
       <c r="D57" t="n">
@@ -1532,7 +1520,7 @@
       <c r="B58" t="n">
         <v>3944</v>
       </c>
-      <c r="C58" s="2" t="n">
+      <c r="C58" s="1" t="n">
         <v>45993.84027777778</v>
       </c>
       <c r="D58" t="n">
@@ -1551,7 +1539,7 @@
       <c r="B59" t="n">
         <v>3944</v>
       </c>
-      <c r="C59" s="2" t="n">
+      <c r="C59" s="1" t="n">
         <v>45993.84375</v>
       </c>
       <c r="D59" t="n">
@@ -1570,7 +1558,7 @@
       <c r="B60" t="n">
         <v>3944</v>
       </c>
-      <c r="C60" s="2" t="n">
+      <c r="C60" s="1" t="n">
         <v>45993.84722222222</v>
       </c>
       <c r="D60" t="n">
@@ -1589,7 +1577,7 @@
       <c r="B61" t="n">
         <v>3944</v>
       </c>
-      <c r="C61" s="2" t="n">
+      <c r="C61" s="1" t="n">
         <v>45993.85069444445</v>
       </c>
       <c r="D61" t="n">
@@ -1608,7 +1596,7 @@
       <c r="B62" t="n">
         <v>3944</v>
       </c>
-      <c r="C62" s="2" t="n">
+      <c r="C62" s="1" t="n">
         <v>45993.85416666666</v>
       </c>
       <c r="D62" t="n">
@@ -1627,7 +1615,7 @@
       <c r="B63" t="n">
         <v>3944</v>
       </c>
-      <c r="C63" s="2" t="n">
+      <c r="C63" s="1" t="n">
         <v>45993.85763888889</v>
       </c>
       <c r="D63" t="n">
@@ -1646,7 +1634,7 @@
       <c r="B64" t="n">
         <v>3944</v>
       </c>
-      <c r="C64" s="2" t="n">
+      <c r="C64" s="1" t="n">
         <v>45993.86111111111</v>
       </c>
       <c r="D64" t="n">
@@ -1665,7 +1653,7 @@
       <c r="B65" t="n">
         <v>3944</v>
       </c>
-      <c r="C65" s="2" t="n">
+      <c r="C65" s="1" t="n">
         <v>45993.86458333334</v>
       </c>
       <c r="D65" t="n">
@@ -1684,7 +1672,7 @@
       <c r="B66" t="n">
         <v>3944</v>
       </c>
-      <c r="C66" s="2" t="n">
+      <c r="C66" s="1" t="n">
         <v>45993.86805555555</v>
       </c>
       <c r="D66" t="n">
@@ -1703,7 +1691,7 @@
       <c r="B67" t="n">
         <v>3944</v>
       </c>
-      <c r="C67" s="2" t="n">
+      <c r="C67" s="1" t="n">
         <v>45993.87152777778</v>
       </c>
       <c r="D67" t="n">
@@ -1722,7 +1710,7 @@
       <c r="B68" t="n">
         <v>3944</v>
       </c>
-      <c r="C68" s="2" t="n">
+      <c r="C68" s="1" t="n">
         <v>45993.875</v>
       </c>
       <c r="D68" t="n">
@@ -1741,7 +1729,7 @@
       <c r="B69" t="n">
         <v>3944</v>
       </c>
-      <c r="C69" s="2" t="n">
+      <c r="C69" s="1" t="n">
         <v>45993.87847222222</v>
       </c>
       <c r="D69" t="n">
@@ -1760,7 +1748,7 @@
       <c r="B70" t="n">
         <v>3944</v>
       </c>
-      <c r="C70" s="2" t="n">
+      <c r="C70" s="1" t="n">
         <v>45993.88194444445</v>
       </c>
       <c r="D70" t="n">
@@ -1779,7 +1767,7 @@
       <c r="B71" t="n">
         <v>3944</v>
       </c>
-      <c r="C71" s="2" t="n">
+      <c r="C71" s="1" t="n">
         <v>45993.88541666666</v>
       </c>
       <c r="D71" t="n">
@@ -1798,7 +1786,7 @@
       <c r="B72" t="n">
         <v>3944</v>
       </c>
-      <c r="C72" s="2" t="n">
+      <c r="C72" s="1" t="n">
         <v>45993.88888888889</v>
       </c>
       <c r="D72" t="n">
@@ -1817,7 +1805,7 @@
       <c r="B73" t="n">
         <v>3944</v>
       </c>
-      <c r="C73" s="2" t="n">
+      <c r="C73" s="1" t="n">
         <v>45993.89236111111</v>
       </c>
       <c r="D73" t="n">
@@ -1836,7 +1824,7 @@
       <c r="B74" t="n">
         <v>3944</v>
       </c>
-      <c r="C74" s="2" t="n">
+      <c r="C74" s="1" t="n">
         <v>45993.89583333334</v>
       </c>
       <c r="D74" t="n">
@@ -1855,7 +1843,7 @@
       <c r="B75" t="n">
         <v>3944</v>
       </c>
-      <c r="C75" s="2" t="n">
+      <c r="C75" s="1" t="n">
         <v>45993.89930555555</v>
       </c>
       <c r="D75" t="n">
@@ -1874,7 +1862,7 @@
       <c r="B76" t="n">
         <v>3944</v>
       </c>
-      <c r="C76" s="2" t="n">
+      <c r="C76" s="1" t="n">
         <v>45993.90277777778</v>
       </c>
       <c r="D76" t="n">
@@ -1893,7 +1881,7 @@
       <c r="B77" t="n">
         <v>3944</v>
       </c>
-      <c r="C77" s="2" t="n">
+      <c r="C77" s="1" t="n">
         <v>45993.90625</v>
       </c>
       <c r="D77" t="n">
@@ -1912,7 +1900,7 @@
       <c r="B78" t="n">
         <v>3944</v>
       </c>
-      <c r="C78" s="2" t="n">
+      <c r="C78" s="1" t="n">
         <v>45993.90972222222</v>
       </c>
       <c r="D78" t="n">
@@ -1931,7 +1919,7 @@
       <c r="B79" t="n">
         <v>3944</v>
       </c>
-      <c r="C79" s="2" t="n">
+      <c r="C79" s="1" t="n">
         <v>45993.91319444445</v>
       </c>
       <c r="D79" t="n">
@@ -1950,7 +1938,7 @@
       <c r="B80" t="n">
         <v>3944</v>
       </c>
-      <c r="C80" s="2" t="n">
+      <c r="C80" s="1" t="n">
         <v>45993.91666666666</v>
       </c>
       <c r="D80" t="n">
@@ -1969,7 +1957,7 @@
       <c r="B81" t="n">
         <v>3944</v>
       </c>
-      <c r="C81" s="2" t="n">
+      <c r="C81" s="1" t="n">
         <v>45993.92013888889</v>
       </c>
       <c r="D81" t="n">
@@ -1988,7 +1976,7 @@
       <c r="B82" t="n">
         <v>3944</v>
       </c>
-      <c r="C82" s="2" t="n">
+      <c r="C82" s="1" t="n">
         <v>45993.92361111111</v>
       </c>
       <c r="D82" t="n">
@@ -2007,7 +1995,7 @@
       <c r="B83" t="n">
         <v>3944</v>
       </c>
-      <c r="C83" s="2" t="n">
+      <c r="C83" s="1" t="n">
         <v>45993.92708333334</v>
       </c>
       <c r="D83" t="n">
@@ -2026,7 +2014,7 @@
       <c r="B84" t="n">
         <v>3944</v>
       </c>
-      <c r="C84" s="2" t="n">
+      <c r="C84" s="1" t="n">
         <v>45993.93055555555</v>
       </c>
       <c r="D84" t="n">
@@ -2045,7 +2033,7 @@
       <c r="B85" t="n">
         <v>3944</v>
       </c>
-      <c r="C85" s="2" t="n">
+      <c r="C85" s="1" t="n">
         <v>45993.93402777778</v>
       </c>
       <c r="D85" t="n">
@@ -2064,7 +2052,7 @@
       <c r="B86" t="n">
         <v>3944</v>
       </c>
-      <c r="C86" s="2" t="n">
+      <c r="C86" s="1" t="n">
         <v>45993.9375</v>
       </c>
       <c r="D86" t="n">
@@ -2083,7 +2071,7 @@
       <c r="B87" t="n">
         <v>3944</v>
       </c>
-      <c r="C87" s="2" t="n">
+      <c r="C87" s="1" t="n">
         <v>45993.94097222222</v>
       </c>
       <c r="D87" t="n">
@@ -2102,7 +2090,7 @@
       <c r="B88" t="n">
         <v>3944</v>
       </c>
-      <c r="C88" s="2" t="n">
+      <c r="C88" s="1" t="n">
         <v>45993.94444444445</v>
       </c>
       <c r="D88" t="n">
@@ -2121,7 +2109,7 @@
       <c r="B89" t="n">
         <v>3944</v>
       </c>
-      <c r="C89" s="2" t="n">
+      <c r="C89" s="1" t="n">
         <v>45993.94791666666</v>
       </c>
       <c r="D89" t="n">
@@ -2140,7 +2128,7 @@
       <c r="B90" t="n">
         <v>3944</v>
       </c>
-      <c r="C90" s="2" t="n">
+      <c r="C90" s="1" t="n">
         <v>45993.95138888889</v>
       </c>
       <c r="D90" t="n">
@@ -2159,7 +2147,7 @@
       <c r="B91" t="n">
         <v>3944</v>
       </c>
-      <c r="C91" s="2" t="n">
+      <c r="C91" s="1" t="n">
         <v>45993.95486111111</v>
       </c>
       <c r="D91" t="n">
@@ -2178,7 +2166,7 @@
       <c r="B92" t="n">
         <v>3944</v>
       </c>
-      <c r="C92" s="2" t="n">
+      <c r="C92" s="1" t="n">
         <v>45993.95833333334</v>
       </c>
       <c r="D92" t="n">
@@ -2197,7 +2185,7 @@
       <c r="B93" t="n">
         <v>3944</v>
       </c>
-      <c r="C93" s="2" t="n">
+      <c r="C93" s="1" t="n">
         <v>45993.96180555555</v>
       </c>
       <c r="D93" t="n">
@@ -2216,7 +2204,7 @@
       <c r="B94" t="n">
         <v>3944</v>
       </c>
-      <c r="C94" s="2" t="n">
+      <c r="C94" s="1" t="n">
         <v>45993.96527777778</v>
       </c>
       <c r="D94" t="n">
@@ -2235,7 +2223,7 @@
       <c r="B95" t="n">
         <v>3944</v>
       </c>
-      <c r="C95" s="2" t="n">
+      <c r="C95" s="1" t="n">
         <v>45993.96875</v>
       </c>
       <c r="D95" t="n">
@@ -2254,7 +2242,7 @@
       <c r="B96" t="n">
         <v>3944</v>
       </c>
-      <c r="C96" s="2" t="n">
+      <c r="C96" s="1" t="n">
         <v>45993.97222222222</v>
       </c>
       <c r="D96" t="n">
@@ -2273,7 +2261,7 @@
       <c r="B97" t="n">
         <v>3944</v>
       </c>
-      <c r="C97" s="2" t="n">
+      <c r="C97" s="1" t="n">
         <v>45993.97569444445</v>
       </c>
       <c r="D97" t="n">
@@ -2292,7 +2280,7 @@
       <c r="B98" t="n">
         <v>3944</v>
       </c>
-      <c r="C98" s="2" t="n">
+      <c r="C98" s="1" t="n">
         <v>45993.97916666666</v>
       </c>
       <c r="D98" t="n">
@@ -2311,7 +2299,7 @@
       <c r="B99" t="n">
         <v>3944</v>
       </c>
-      <c r="C99" s="2" t="n">
+      <c r="C99" s="1" t="n">
         <v>45993.98263888889</v>
       </c>
       <c r="D99" t="n">
@@ -2330,7 +2318,7 @@
       <c r="B100" t="n">
         <v>3944</v>
       </c>
-      <c r="C100" s="2" t="n">
+      <c r="C100" s="1" t="n">
         <v>45993.98611111111</v>
       </c>
       <c r="D100" t="n">
@@ -2349,7 +2337,7 @@
       <c r="B101" t="n">
         <v>3944</v>
       </c>
-      <c r="C101" s="2" t="n">
+      <c r="C101" s="1" t="n">
         <v>45993.98958333334</v>
       </c>
       <c r="D101" t="n">
@@ -2368,7 +2356,7 @@
       <c r="B102" t="n">
         <v>3944</v>
       </c>
-      <c r="C102" s="2" t="n">
+      <c r="C102" s="1" t="n">
         <v>45993.99305555555</v>
       </c>
       <c r="D102" t="n">
@@ -2387,7 +2375,7 @@
       <c r="B103" t="n">
         <v>3944</v>
       </c>
-      <c r="C103" s="2" t="n">
+      <c r="C103" s="1" t="n">
         <v>45993.99652777778</v>
       </c>
       <c r="D103" t="n">
@@ -2406,7 +2394,7 @@
       <c r="B104" t="n">
         <v>3944</v>
       </c>
-      <c r="C104" s="2" t="n">
+      <c r="C104" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="D104" t="n">
@@ -2425,7 +2413,7 @@
       <c r="B105" t="n">
         <v>3944</v>
       </c>
-      <c r="C105" s="2" t="n">
+      <c r="C105" s="1" t="n">
         <v>45994.00347222222</v>
       </c>
       <c r="D105" t="n">
@@ -2444,7 +2432,7 @@
       <c r="B106" t="n">
         <v>3944</v>
       </c>
-      <c r="C106" s="2" t="n">
+      <c r="C106" s="1" t="n">
         <v>45994.00694444445</v>
       </c>
       <c r="D106" t="n">
@@ -2463,7 +2451,7 @@
       <c r="B107" t="n">
         <v>3944</v>
       </c>
-      <c r="C107" s="2" t="n">
+      <c r="C107" s="1" t="n">
         <v>45994.01041666666</v>
       </c>
       <c r="D107" t="n">
@@ -2482,7 +2470,7 @@
       <c r="B108" t="n">
         <v>3944</v>
       </c>
-      <c r="C108" s="2" t="n">
+      <c r="C108" s="1" t="n">
         <v>45994.01388888889</v>
       </c>
       <c r="D108" t="n">
@@ -2501,7 +2489,7 @@
       <c r="B109" t="n">
         <v>3944</v>
       </c>
-      <c r="C109" s="2" t="n">
+      <c r="C109" s="1" t="n">
         <v>45994.01736111111</v>
       </c>
       <c r="D109" t="n">
@@ -2520,7 +2508,7 @@
       <c r="B110" t="n">
         <v>3944</v>
       </c>
-      <c r="C110" s="2" t="n">
+      <c r="C110" s="1" t="n">
         <v>45994.02083333334</v>
       </c>
       <c r="D110" t="n">
@@ -2539,7 +2527,7 @@
       <c r="B111" t="n">
         <v>3944</v>
       </c>
-      <c r="C111" s="2" t="n">
+      <c r="C111" s="1" t="n">
         <v>45994.02430555555</v>
       </c>
       <c r="D111" t="n">
@@ -2558,7 +2546,7 @@
       <c r="B112" t="n">
         <v>3944</v>
       </c>
-      <c r="C112" s="2" t="n">
+      <c r="C112" s="1" t="n">
         <v>45994.02777777778</v>
       </c>
       <c r="D112" t="n">
@@ -2577,7 +2565,7 @@
       <c r="B113" t="n">
         <v>3944</v>
       </c>
-      <c r="C113" s="2" t="n">
+      <c r="C113" s="1" t="n">
         <v>45994.03125</v>
       </c>
       <c r="D113" t="n">
@@ -2596,7 +2584,7 @@
       <c r="B114" t="n">
         <v>3944</v>
       </c>
-      <c r="C114" s="2" t="n">
+      <c r="C114" s="1" t="n">
         <v>45994.03472222222</v>
       </c>
       <c r="D114" t="n">
@@ -2615,7 +2603,7 @@
       <c r="B115" t="n">
         <v>3944</v>
       </c>
-      <c r="C115" s="2" t="n">
+      <c r="C115" s="1" t="n">
         <v>45994.03819444445</v>
       </c>
       <c r="D115" t="n">
@@ -2634,7 +2622,7 @@
       <c r="B116" t="n">
         <v>3944</v>
       </c>
-      <c r="C116" s="2" t="n">
+      <c r="C116" s="1" t="n">
         <v>45994.04166666666</v>
       </c>
       <c r="D116" t="n">
@@ -2653,7 +2641,7 @@
       <c r="B117" t="n">
         <v>3944</v>
       </c>
-      <c r="C117" s="2" t="n">
+      <c r="C117" s="1" t="n">
         <v>45994.04513888889</v>
       </c>
       <c r="D117" t="n">
@@ -2672,7 +2660,7 @@
       <c r="B118" t="n">
         <v>3944</v>
       </c>
-      <c r="C118" s="2" t="n">
+      <c r="C118" s="1" t="n">
         <v>45994.04861111111</v>
       </c>
       <c r="D118" t="n">
@@ -2691,7 +2679,7 @@
       <c r="B119" t="n">
         <v>3944</v>
       </c>
-      <c r="C119" s="2" t="n">
+      <c r="C119" s="1" t="n">
         <v>45994.05208333334</v>
       </c>
       <c r="D119" t="n">
@@ -2710,7 +2698,7 @@
       <c r="B120" t="n">
         <v>3944</v>
       </c>
-      <c r="C120" s="2" t="n">
+      <c r="C120" s="1" t="n">
         <v>45994.05555555555</v>
       </c>
       <c r="D120" t="n">
@@ -2729,7 +2717,7 @@
       <c r="B121" t="n">
         <v>3944</v>
       </c>
-      <c r="C121" s="2" t="n">
+      <c r="C121" s="1" t="n">
         <v>45994.05902777778</v>
       </c>
       <c r="D121" t="n">
@@ -2748,7 +2736,7 @@
       <c r="B122" t="n">
         <v>3944</v>
       </c>
-      <c r="C122" s="2" t="n">
+      <c r="C122" s="1" t="n">
         <v>45994.0625</v>
       </c>
       <c r="D122" t="n">
@@ -2767,7 +2755,7 @@
       <c r="B123" t="n">
         <v>3944</v>
       </c>
-      <c r="C123" s="2" t="n">
+      <c r="C123" s="1" t="n">
         <v>45994.06597222222</v>
       </c>
       <c r="D123" t="n">
@@ -2786,7 +2774,7 @@
       <c r="B124" t="n">
         <v>3944</v>
       </c>
-      <c r="C124" s="2" t="n">
+      <c r="C124" s="1" t="n">
         <v>45994.06944444445</v>
       </c>
       <c r="D124" t="n">
@@ -2805,7 +2793,7 @@
       <c r="B125" t="n">
         <v>3944</v>
       </c>
-      <c r="C125" s="2" t="n">
+      <c r="C125" s="1" t="n">
         <v>45994.07291666666</v>
       </c>
       <c r="D125" t="n">
@@ -2824,7 +2812,7 @@
       <c r="B126" t="n">
         <v>3944</v>
       </c>
-      <c r="C126" s="2" t="n">
+      <c r="C126" s="1" t="n">
         <v>45994.07638888889</v>
       </c>
       <c r="D126" t="n">
@@ -2843,7 +2831,7 @@
       <c r="B127" t="n">
         <v>3944</v>
       </c>
-      <c r="C127" s="2" t="n">
+      <c r="C127" s="1" t="n">
         <v>45994.07986111111</v>
       </c>
       <c r="D127" t="n">
@@ -2862,7 +2850,7 @@
       <c r="B128" t="n">
         <v>3944</v>
       </c>
-      <c r="C128" s="2" t="n">
+      <c r="C128" s="1" t="n">
         <v>45994.08333333334</v>
       </c>
       <c r="D128" t="n">
@@ -2881,7 +2869,7 @@
       <c r="B129" t="n">
         <v>3944</v>
       </c>
-      <c r="C129" s="2" t="n">
+      <c r="C129" s="1" t="n">
         <v>45994.08680555555</v>
       </c>
       <c r="D129" t="n">
@@ -2900,7 +2888,7 @@
       <c r="B130" t="n">
         <v>3944</v>
       </c>
-      <c r="C130" s="2" t="n">
+      <c r="C130" s="1" t="n">
         <v>45994.09027777778</v>
       </c>
       <c r="D130" t="n">
@@ -2919,7 +2907,7 @@
       <c r="B131" t="n">
         <v>3944</v>
       </c>
-      <c r="C131" s="2" t="n">
+      <c r="C131" s="1" t="n">
         <v>45994.09375</v>
       </c>
       <c r="D131" t="n">
@@ -2938,7 +2926,7 @@
       <c r="B132" t="n">
         <v>3944</v>
       </c>
-      <c r="C132" s="2" t="n">
+      <c r="C132" s="1" t="n">
         <v>45994.09722222222</v>
       </c>
       <c r="D132" t="n">
@@ -2957,7 +2945,7 @@
       <c r="B133" t="n">
         <v>3944</v>
       </c>
-      <c r="C133" s="2" t="n">
+      <c r="C133" s="1" t="n">
         <v>45994.10069444445</v>
       </c>
       <c r="D133" t="n">
@@ -2976,7 +2964,7 @@
       <c r="B134" t="n">
         <v>3944</v>
       </c>
-      <c r="C134" s="2" t="n">
+      <c r="C134" s="1" t="n">
         <v>45994.10416666666</v>
       </c>
       <c r="D134" t="n">
@@ -2995,7 +2983,7 @@
       <c r="B135" t="n">
         <v>3944</v>
       </c>
-      <c r="C135" s="2" t="n">
+      <c r="C135" s="1" t="n">
         <v>45994.10763888889</v>
       </c>
       <c r="D135" t="n">
@@ -3014,7 +3002,7 @@
       <c r="B136" t="n">
         <v>3944</v>
       </c>
-      <c r="C136" s="2" t="n">
+      <c r="C136" s="1" t="n">
         <v>45994.11111111111</v>
       </c>
       <c r="D136" t="n">
@@ -3033,7 +3021,7 @@
       <c r="B137" t="n">
         <v>3944</v>
       </c>
-      <c r="C137" s="2" t="n">
+      <c r="C137" s="1" t="n">
         <v>45994.11458333334</v>
       </c>
       <c r="D137" t="n">
@@ -3052,7 +3040,7 @@
       <c r="B138" t="n">
         <v>3944</v>
       </c>
-      <c r="C138" s="2" t="n">
+      <c r="C138" s="1" t="n">
         <v>45994.11805555555</v>
       </c>
       <c r="D138" t="n">
@@ -3071,7 +3059,7 @@
       <c r="B139" t="n">
         <v>3944</v>
       </c>
-      <c r="C139" s="2" t="n">
+      <c r="C139" s="1" t="n">
         <v>45994.12152777778</v>
       </c>
       <c r="D139" t="n">
@@ -3090,7 +3078,7 @@
       <c r="B140" t="n">
         <v>3944</v>
       </c>
-      <c r="C140" s="2" t="n">
+      <c r="C140" s="1" t="n">
         <v>45994.125</v>
       </c>
       <c r="D140" t="n">
@@ -3109,7 +3097,7 @@
       <c r="B141" t="n">
         <v>3944</v>
       </c>
-      <c r="C141" s="2" t="n">
+      <c r="C141" s="1" t="n">
         <v>45994.12847222222</v>
       </c>
       <c r="D141" t="n">
@@ -3128,7 +3116,7 @@
       <c r="B142" t="n">
         <v>3944</v>
       </c>
-      <c r="C142" s="2" t="n">
+      <c r="C142" s="1" t="n">
         <v>45994.13194444445</v>
       </c>
       <c r="D142" t="n">
@@ -3147,7 +3135,7 @@
       <c r="B143" t="n">
         <v>3944</v>
       </c>
-      <c r="C143" s="2" t="n">
+      <c r="C143" s="1" t="n">
         <v>45994.13541666666</v>
       </c>
       <c r="D143" t="n">
@@ -3166,7 +3154,7 @@
       <c r="B144" t="n">
         <v>3944</v>
       </c>
-      <c r="C144" s="2" t="n">
+      <c r="C144" s="1" t="n">
         <v>45994.13888888889</v>
       </c>
       <c r="D144" t="n">
@@ -3185,7 +3173,7 @@
       <c r="B145" t="n">
         <v>3944</v>
       </c>
-      <c r="C145" s="2" t="n">
+      <c r="C145" s="1" t="n">
         <v>45994.14236111111</v>
       </c>
       <c r="D145" t="n">
@@ -3204,7 +3192,7 @@
       <c r="B146" t="n">
         <v>3944</v>
       </c>
-      <c r="C146" s="2" t="n">
+      <c r="C146" s="1" t="n">
         <v>45994.14583333334</v>
       </c>
       <c r="D146" t="n">
@@ -3223,7 +3211,7 @@
       <c r="B147" t="n">
         <v>3944</v>
       </c>
-      <c r="C147" s="2" t="n">
+      <c r="C147" s="1" t="n">
         <v>45994.14930555555</v>
       </c>
       <c r="D147" t="n">
@@ -3242,7 +3230,7 @@
       <c r="B148" t="n">
         <v>3944</v>
       </c>
-      <c r="C148" s="2" t="n">
+      <c r="C148" s="1" t="n">
         <v>45994.15277777778</v>
       </c>
       <c r="D148" t="n">
@@ -3261,7 +3249,7 @@
       <c r="B149" t="n">
         <v>3944</v>
       </c>
-      <c r="C149" s="2" t="n">
+      <c r="C149" s="1" t="n">
         <v>45994.15625</v>
       </c>
       <c r="D149" t="n">
@@ -3280,7 +3268,7 @@
       <c r="B150" t="n">
         <v>3944</v>
       </c>
-      <c r="C150" s="2" t="n">
+      <c r="C150" s="1" t="n">
         <v>45994.15972222222</v>
       </c>
       <c r="D150" t="n">
@@ -3299,7 +3287,7 @@
       <c r="B151" t="n">
         <v>3944</v>
       </c>
-      <c r="C151" s="2" t="n">
+      <c r="C151" s="1" t="n">
         <v>45994.16319444445</v>
       </c>
       <c r="D151" t="n">
@@ -3318,7 +3306,7 @@
       <c r="B152" t="n">
         <v>3944</v>
       </c>
-      <c r="C152" s="2" t="n">
+      <c r="C152" s="1" t="n">
         <v>45994.16666666666</v>
       </c>
       <c r="D152" t="n">
@@ -3337,7 +3325,7 @@
       <c r="B153" t="n">
         <v>3944</v>
       </c>
-      <c r="C153" s="2" t="n">
+      <c r="C153" s="1" t="n">
         <v>45994.17013888889</v>
       </c>
       <c r="D153" t="n">
@@ -3356,7 +3344,7 @@
       <c r="B154" t="n">
         <v>3944</v>
       </c>
-      <c r="C154" s="2" t="n">
+      <c r="C154" s="1" t="n">
         <v>45994.17361111111</v>
       </c>
       <c r="D154" t="n">
@@ -3375,7 +3363,7 @@
       <c r="B155" t="n">
         <v>3944</v>
       </c>
-      <c r="C155" s="2" t="n">
+      <c r="C155" s="1" t="n">
         <v>45994.17708333334</v>
       </c>
       <c r="D155" t="n">
@@ -3394,7 +3382,7 @@
       <c r="B156" t="n">
         <v>3944</v>
       </c>
-      <c r="C156" s="2" t="n">
+      <c r="C156" s="1" t="n">
         <v>45994.18055555555</v>
       </c>
       <c r="D156" t="n">
@@ -3413,7 +3401,7 @@
       <c r="B157" t="n">
         <v>3944</v>
       </c>
-      <c r="C157" s="2" t="n">
+      <c r="C157" s="1" t="n">
         <v>45994.18402777778</v>
       </c>
       <c r="D157" t="n">
@@ -3432,7 +3420,7 @@
       <c r="B158" t="n">
         <v>3944</v>
       </c>
-      <c r="C158" s="2" t="n">
+      <c r="C158" s="1" t="n">
         <v>45994.1875</v>
       </c>
       <c r="D158" t="n">
@@ -3451,7 +3439,7 @@
       <c r="B159" t="n">
         <v>3944</v>
       </c>
-      <c r="C159" s="2" t="n">
+      <c r="C159" s="1" t="n">
         <v>45994.19097222222</v>
       </c>
       <c r="D159" t="n">
@@ -3470,7 +3458,7 @@
       <c r="B160" t="n">
         <v>3944</v>
       </c>
-      <c r="C160" s="2" t="n">
+      <c r="C160" s="1" t="n">
         <v>45994.19444444445</v>
       </c>
       <c r="D160" t="n">
@@ -3489,7 +3477,7 @@
       <c r="B161" t="n">
         <v>3944</v>
       </c>
-      <c r="C161" s="2" t="n">
+      <c r="C161" s="1" t="n">
         <v>45994.19791666666</v>
       </c>
       <c r="D161" t="n">
@@ -3508,7 +3496,7 @@
       <c r="B162" t="n">
         <v>3944</v>
       </c>
-      <c r="C162" s="2" t="n">
+      <c r="C162" s="1" t="n">
         <v>45994.20138888889</v>
       </c>
       <c r="D162" t="n">
@@ -3527,7 +3515,7 @@
       <c r="B163" t="n">
         <v>3944</v>
       </c>
-      <c r="C163" s="2" t="n">
+      <c r="C163" s="1" t="n">
         <v>45994.20486111111</v>
       </c>
       <c r="D163" t="n">
@@ -3546,7 +3534,7 @@
       <c r="B164" t="n">
         <v>3944</v>
       </c>
-      <c r="C164" s="2" t="n">
+      <c r="C164" s="1" t="n">
         <v>45994.20833333334</v>
       </c>
       <c r="D164" t="n">
@@ -3565,7 +3553,7 @@
       <c r="B165" t="n">
         <v>3944</v>
       </c>
-      <c r="C165" s="2" t="n">
+      <c r="C165" s="1" t="n">
         <v>45994.21180555555</v>
       </c>
       <c r="D165" t="n">
@@ -3584,7 +3572,7 @@
       <c r="B166" t="n">
         <v>3944</v>
       </c>
-      <c r="C166" s="2" t="n">
+      <c r="C166" s="1" t="n">
         <v>45994.21527777778</v>
       </c>
       <c r="D166" t="n">
@@ -3603,7 +3591,7 @@
       <c r="B167" t="n">
         <v>3944</v>
       </c>
-      <c r="C167" s="2" t="n">
+      <c r="C167" s="1" t="n">
         <v>45994.21875</v>
       </c>
       <c r="D167" t="n">
@@ -3622,7 +3610,7 @@
       <c r="B168" t="n">
         <v>3944</v>
       </c>
-      <c r="C168" s="2" t="n">
+      <c r="C168" s="1" t="n">
         <v>45994.22222222222</v>
       </c>
       <c r="D168" t="n">
@@ -3641,7 +3629,7 @@
       <c r="B169" t="n">
         <v>3944</v>
       </c>
-      <c r="C169" s="2" t="n">
+      <c r="C169" s="1" t="n">
         <v>45994.22569444445</v>
       </c>
       <c r="D169" t="n">
@@ -3660,7 +3648,7 @@
       <c r="B170" t="n">
         <v>3944</v>
       </c>
-      <c r="C170" s="2" t="n">
+      <c r="C170" s="1" t="n">
         <v>45994.22916666666</v>
       </c>
       <c r="D170" t="n">
@@ -3679,7 +3667,7 @@
       <c r="B171" t="n">
         <v>3944</v>
       </c>
-      <c r="C171" s="2" t="n">
+      <c r="C171" s="1" t="n">
         <v>45994.23263888889</v>
       </c>
       <c r="D171" t="n">
@@ -3698,7 +3686,7 @@
       <c r="B172" t="n">
         <v>3944</v>
       </c>
-      <c r="C172" s="2" t="n">
+      <c r="C172" s="1" t="n">
         <v>45994.23611111111</v>
       </c>
       <c r="D172" t="n">
@@ -3717,7 +3705,7 @@
       <c r="B173" t="n">
         <v>3944</v>
       </c>
-      <c r="C173" s="2" t="n">
+      <c r="C173" s="1" t="n">
         <v>45994.23958333334</v>
       </c>
       <c r="D173" t="n">
@@ -3736,7 +3724,7 @@
       <c r="B174" t="n">
         <v>3944</v>
       </c>
-      <c r="C174" s="2" t="n">
+      <c r="C174" s="1" t="n">
         <v>45994.24305555555</v>
       </c>
       <c r="D174" t="n">
@@ -3755,7 +3743,7 @@
       <c r="B175" t="n">
         <v>3944</v>
       </c>
-      <c r="C175" s="2" t="n">
+      <c r="C175" s="1" t="n">
         <v>45994.24652777778</v>
       </c>
       <c r="D175" t="n">
@@ -3774,7 +3762,7 @@
       <c r="B176" t="n">
         <v>3944</v>
       </c>
-      <c r="C176" s="2" t="n">
+      <c r="C176" s="1" t="n">
         <v>45994.25</v>
       </c>
       <c r="D176" t="n">
@@ -3793,7 +3781,7 @@
       <c r="B177" t="n">
         <v>3944</v>
       </c>
-      <c r="C177" s="2" t="n">
+      <c r="C177" s="1" t="n">
         <v>45994.25347222222</v>
       </c>
       <c r="D177" t="n">
@@ -3812,7 +3800,7 @@
       <c r="B178" t="n">
         <v>3944</v>
       </c>
-      <c r="C178" s="2" t="n">
+      <c r="C178" s="1" t="n">
         <v>45994.25694444445</v>
       </c>
       <c r="D178" t="n">
@@ -3831,7 +3819,7 @@
       <c r="B179" t="n">
         <v>3944</v>
       </c>
-      <c r="C179" s="2" t="n">
+      <c r="C179" s="1" t="n">
         <v>45994.26041666666</v>
       </c>
       <c r="D179" t="n">
@@ -3850,7 +3838,7 @@
       <c r="B180" t="n">
         <v>3944</v>
       </c>
-      <c r="C180" s="2" t="n">
+      <c r="C180" s="1" t="n">
         <v>45994.26388888889</v>
       </c>
       <c r="D180" t="n">
@@ -3869,7 +3857,7 @@
       <c r="B181" t="n">
         <v>3944</v>
       </c>
-      <c r="C181" s="2" t="n">
+      <c r="C181" s="1" t="n">
         <v>45994.26736111111</v>
       </c>
       <c r="D181" t="n">
@@ -3888,7 +3876,7 @@
       <c r="B182" t="n">
         <v>3944</v>
       </c>
-      <c r="C182" s="2" t="n">
+      <c r="C182" s="1" t="n">
         <v>45994.27083333334</v>
       </c>
       <c r="D182" t="n">
@@ -3907,7 +3895,7 @@
       <c r="B183" t="n">
         <v>3944</v>
       </c>
-      <c r="C183" s="2" t="n">
+      <c r="C183" s="1" t="n">
         <v>45994.27430555555</v>
       </c>
       <c r="D183" t="n">
@@ -3926,7 +3914,7 @@
       <c r="B184" t="n">
         <v>3944</v>
       </c>
-      <c r="C184" s="2" t="n">
+      <c r="C184" s="1" t="n">
         <v>45994.27777777778</v>
       </c>
       <c r="D184" t="n">
@@ -3945,7 +3933,7 @@
       <c r="B185" t="n">
         <v>3944</v>
       </c>
-      <c r="C185" s="2" t="n">
+      <c r="C185" s="1" t="n">
         <v>45994.28125</v>
       </c>
       <c r="D185" t="n">
@@ -3964,7 +3952,7 @@
       <c r="B186" t="n">
         <v>3944</v>
       </c>
-      <c r="C186" s="2" t="n">
+      <c r="C186" s="1" t="n">
         <v>45994.28472222222</v>
       </c>
       <c r="D186" t="n">
@@ -3983,7 +3971,7 @@
       <c r="B187" t="n">
         <v>3944</v>
       </c>
-      <c r="C187" s="2" t="n">
+      <c r="C187" s="1" t="n">
         <v>45994.28819444445</v>
       </c>
       <c r="D187" t="n">
@@ -4002,7 +3990,7 @@
       <c r="B188" t="n">
         <v>3944</v>
       </c>
-      <c r="C188" s="2" t="n">
+      <c r="C188" s="1" t="n">
         <v>45994.29166666666</v>
       </c>
       <c r="D188" t="n">
@@ -4021,7 +4009,7 @@
       <c r="B189" t="n">
         <v>3944</v>
       </c>
-      <c r="C189" s="2" t="n">
+      <c r="C189" s="1" t="n">
         <v>45994.29513888889</v>
       </c>
       <c r="D189" t="n">
@@ -4040,7 +4028,7 @@
       <c r="B190" t="n">
         <v>3944</v>
       </c>
-      <c r="C190" s="2" t="n">
+      <c r="C190" s="1" t="n">
         <v>45994.29861111111</v>
       </c>
       <c r="D190" t="n">
@@ -4059,7 +4047,7 @@
       <c r="B191" t="n">
         <v>3944</v>
       </c>
-      <c r="C191" s="2" t="n">
+      <c r="C191" s="1" t="n">
         <v>45994.30208333334</v>
       </c>
       <c r="D191" t="n">
@@ -4078,7 +4066,7 @@
       <c r="B192" t="n">
         <v>3944</v>
       </c>
-      <c r="C192" s="2" t="n">
+      <c r="C192" s="1" t="n">
         <v>45994.30555555555</v>
       </c>
       <c r="D192" t="n">
@@ -4097,7 +4085,7 @@
       <c r="B193" t="n">
         <v>3944</v>
       </c>
-      <c r="C193" s="2" t="n">
+      <c r="C193" s="1" t="n">
         <v>45994.30902777778</v>
       </c>
       <c r="D193" t="n">
@@ -4116,7 +4104,7 @@
       <c r="B194" t="n">
         <v>3944</v>
       </c>
-      <c r="C194" s="2" t="n">
+      <c r="C194" s="1" t="n">
         <v>45994.3125</v>
       </c>
       <c r="D194" t="n">
@@ -4135,7 +4123,7 @@
       <c r="B195" t="n">
         <v>3944</v>
       </c>
-      <c r="C195" s="2" t="n">
+      <c r="C195" s="1" t="n">
         <v>45994.31597222222</v>
       </c>
       <c r="D195" t="n">
@@ -4154,7 +4142,7 @@
       <c r="B196" t="n">
         <v>3944</v>
       </c>
-      <c r="C196" s="2" t="n">
+      <c r="C196" s="1" t="n">
         <v>45994.31944444445</v>
       </c>
       <c r="D196" t="n">
@@ -4173,7 +4161,7 @@
       <c r="B197" t="n">
         <v>3944</v>
       </c>
-      <c r="C197" s="2" t="n">
+      <c r="C197" s="1" t="n">
         <v>45994.32291666666</v>
       </c>
       <c r="D197" t="n">
@@ -4192,7 +4180,7 @@
       <c r="B198" t="n">
         <v>3944</v>
       </c>
-      <c r="C198" s="2" t="n">
+      <c r="C198" s="1" t="n">
         <v>45994.32638888889</v>
       </c>
       <c r="D198" t="n">
@@ -4211,7 +4199,7 @@
       <c r="B199" t="n">
         <v>3944</v>
       </c>
-      <c r="C199" s="2" t="n">
+      <c r="C199" s="1" t="n">
         <v>45994.32986111111</v>
       </c>
       <c r="D199" t="n">
@@ -4230,7 +4218,7 @@
       <c r="B200" t="n">
         <v>3944</v>
       </c>
-      <c r="C200" s="2" t="n">
+      <c r="C200" s="1" t="n">
         <v>45994.33333333334</v>
       </c>
       <c r="D200" t="n">
@@ -4249,7 +4237,7 @@
       <c r="B201" t="n">
         <v>3944</v>
       </c>
-      <c r="C201" s="2" t="n">
+      <c r="C201" s="1" t="n">
         <v>45994.33680555555</v>
       </c>
       <c r="D201" t="n">
@@ -4268,7 +4256,7 @@
       <c r="B202" t="n">
         <v>3944</v>
       </c>
-      <c r="C202" s="2" t="n">
+      <c r="C202" s="1" t="n">
         <v>45994.34027777778</v>
       </c>
       <c r="D202" t="n">
@@ -4287,7 +4275,7 @@
       <c r="B203" t="n">
         <v>3944</v>
       </c>
-      <c r="C203" s="2" t="n">
+      <c r="C203" s="1" t="n">
         <v>45994.34375</v>
       </c>
       <c r="D203" t="n">

</xml_diff>